<commit_message>
Update itinerary with new bookings and refine conventions
- Expand CLAUDE.md with retention rules, <...> placeholder handling,
  positional inference, activity routing, and Tips row spec
- Add Bounce (Prague) and GetYourGuide booking confirmations
- Sync info_notes.txt with latest bookings
- Regenerate xlsx + pdf outputs (timestamped versions retained)
- Remove obsolete trip-notes.txt

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/euro_2026_itinerary.xlsx
+++ b/output/euro_2026_itinerary.xlsx
@@ -36,7 +36,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -60,12 +60,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00E4D7F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -100,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -118,6 +123,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -485,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18.7" customWidth="1" min="1" max="1"/>
@@ -581,7 +589,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Ninoy Aquino International Airport (Manila)</t>
+          <t>Ninoy Aquino International Airport (Manila) — 21:25</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -695,32 +703,20 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Lodging (Airbnb)</t>
+          <t>Tips</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Margaretengürtel 6, 1050 Wien, Austria</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>Check-in: 2026-05-18</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>Check-out: 2026-05-22</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>4 nights</t>
-        </is>
-      </c>
+          <t>Wiener Linien 72-hour pass (~€17.10) — U-Bahn + tram + bus across all zones</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr"/>
+      <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>Google Maps: https://maps.app.goo.gl/bAQYMCvSrB3vRvXn7</t>
+          <t>Attractions: Sisi Ticket (€44) bundles Hofburg Imperial Apartments + Schönbrunn + Imperial Furniture; Vienna Pass for heavy sightseeing; Vienna State Opera standing-room (€4-15) | Explore: Sachertorte at Café Sacher, Wiener Schnitzel at Figlmüller, Naschmarkt food market, classic coffeehouses (Café Central, Hawelka)</t>
         </is>
       </c>
     </row>
@@ -737,7 +733,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Evening</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -752,509 +748,1393 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Walk around Stephansplatz; visit St. Stephen's Cathedral</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr"/>
-      <c r="I6" s="5" t="inlineStr"/>
+          <t>St. Stephen's Cathedral (Stephansdom), Stephansplatz 3, 1010 Wien, Austria</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>From: Wiednergürtel 48/IV, 1040 Wien (Bounce Luggage)</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>10:10 (est.)</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>10 min</t>
+        </is>
+      </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>Evening activity after Airbnb check-in</t>
+          <t>Walk 3 min to Südtiroler Platz → U-Bahn U1 to Stephansplatz | https://www.google.com/maps/dir/?api=1&amp;origin=Wiednerg%C3%BCrtel%2048/IV%2C%201040%20Wien&amp;destination=Stephansplatz%203%2C%201010%20Wien&amp;travelmode=transit</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-20</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Wed</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>07:34</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>Vienna → Budapest</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>Train</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>RegioJet RJ 1065</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>Vienna Central Train Station — 07:34</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>Budapest Déli — 10:14</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>2h 40m</t>
-        </is>
-      </c>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>Trainline: https://app.trainline.com/QrswMpOb12b</t>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Vienna</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Ausgrabungen Michaelerplatz, Michaelerplatz, 1010 Wien, Austria (open-air Roman &amp; medieval excavations)</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>From: Stephansplatz 3, 1010 Wien (St. Stephen's Cathedral)</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>11:35 (est.)</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Walk via Graben &amp; Kohlmarkt | https://www.google.com/maps/dir/?api=1&amp;origin=Stephansplatz%203%2C%201010%20Wien&amp;destination=Michaelerplatz%2C%201010%20Wien&amp;travelmode=walking</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Vienna</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Lodging (Airbnb)</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Margaretengürtel 6, 1050 Wien, Austria</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Check-in: 2026-05-18 16:30</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>Check-out: 2026-05-22</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>4 nights</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>Google Maps: https://maps.app.goo.gl/bAQYMCvSrB3vRvXn7</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Vienna</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>GuruWalk 'Free Tour Vienna — Part 1, the highlights' (2-hour free/tip-based walking tour; stops include Heldenplatz, Hofburg, Stephansdom). Meeting point: Karlsplatz U-Bahn station, 1010 Wien, Austria</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>From: Margaretengürtel 6, 1050 Wien (Airbnb)</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>10:10 (est.)</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>25 min</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>Tour 10:15–12:15. Booking: https://www.guruwalk.com/walks/36416-free-tour-vienna-part-1-the-highlights | U-Bahn U4 from Margaretengürtel → Karlsplatz | https://www.google.com/maps/dir/?api=1&amp;origin=Margareteng%C3%BCrtel%206%2C%201050%20Wien&amp;destination=Karlsplatz%20U-Bahn%2C%201010%20Wien&amp;travelmode=transit</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Vienna</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Belvedere Palace (Upper) — Prinz Eugen-Straße 27, 1030 Wien (Klimt's 'The Kiss'; Baroque palace + gardens)</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>From: Karlsplatz / city centre (after walking tour + ~1h lunch break 12:15–13:30)</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>13:45 (est.)</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>15 min</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>Tram D from Karlsplatz → Belvedere (Schloss); allow ~1h lunch between tour end (12:15) and departure | https://www.google.com/maps/dir/?api=1&amp;origin=Karlsplatz%2C%201010%20Wien&amp;destination=Belvedere%20Palace%2C%20Vienna&amp;travelmode=transit</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
           <t>2026-05-20</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Wed</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>07:34</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Vienna → Budapest</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Train</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>RegioJet RJ 1065</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>Vienna Central Train Station — 07:34</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Budapest Déli — 10:14</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>2h 40m</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>Trainline: https://app.trainline.com/QrswMpOb12b</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr"/>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Budapest</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Tips</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>BKV 24-hour ticket (~HUF 2,500 / €6.30) — metro + tram + bus; pair with M2 line from Déli station</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr"/>
+      <c r="H12" s="4" t="inlineStr"/>
+      <c r="I12" s="4" t="inlineStr"/>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>Attractions: Budapest Card (~€36/24h) bundles transit + 30+ sights + 2 thermal baths; Buda Castle district (Fisherman's Bastion outside is free); Széchenyi or Gellért Thermal Baths (bring swimsuit) | Explore: lángos at Karaván Street Food, goulash + kürtőskalács chimney cake, ruin bars in Jewish Quarter (Szimpla Kert), Parliament view from Pest embankment at sunset</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Budapest</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Hungarian Parliament Building (exterior) — Kossuth Lajos tér 1-3, 1055 Budapest</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>From: Budapest Déli (Krisztina körút 37, 1013 Budapest)</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>10:45 (est.)</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>15 min</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>M2 metro Déli → Kossuth tér (direct, ~10 min). 15-min photo stop on Kossuth tér; interior tours need advance booking | https://www.google.com/maps/dir/?api=1&amp;origin=Budapest%20D%C3%A9li%2C%20Krisztina%20k%C3%B6r%C3%BAt%2037%2C%201013%20Budapest&amp;destination=Hungarian%20Parliament%2C%20Kossuth%20Lajos%20t%C3%A9r%201-3%2C%201055%20Budapest&amp;travelmode=transit</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Budapest</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Shoes on the Danube Bank — Id. Antall József rkp., 1054 Budapest (memorial; free, outdoor)</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>From: Hungarian Parliament, Kossuth Lajos tér</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>11:05 (est.)</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>Walk south along Danube embankment | https://www.google.com/maps/dir/?api=1&amp;origin=Kossuth%20Lajos%20t%C3%A9r%2C%20Budapest&amp;destination=Shoes%20on%20the%20Danube%20Bank%2C%20Budapest&amp;travelmode=walking</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Budapest</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>St. Stephen's Basilica — Szent István tér 1, 1051 Budapest (climb the dome ~€4 for panorama)</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>From: Shoes on the Danube Bank</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>11:30 (est.)</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>10 min</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>Walk inland; ~45-min visit | https://www.google.com/maps/dir/?api=1&amp;origin=Shoes%20on%20the%20Danube%20Bank%2C%20Budapest&amp;destination=St.%20Stephen%27s%20Basilica%2C%20Szent%20Istv%C3%A1n%20t%C3%A9r%201%2C%201051%20Budapest&amp;travelmode=walking</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Budapest</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Lunch — Vörösmarty / Erzsébet tér area, 1051 Budapest (suggested: Frici Papa or Belvárosi Disznótoros for goulash, chicken paprikash, kürtőskalács)</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>From: St. Stephen's Basilica</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>12:25 (est.)</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>10 min</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>Walk ~10 min; allow 1h for lunch | https://www.google.com/maps/dir/?api=1&amp;origin=St.%20Stephen%27s%20Basilica%2C%20Budapest&amp;destination=V%C3%B6r%C3%B6smarty%20t%C3%A9r%2C%20Budapest&amp;travelmode=walking</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>13:35</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Budapest</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Buda Castle / Royal Palace courtyards — Szent György tér 2, 1014 Budapest (exterior + viewpoints over Pest)</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>From: Vörösmarty / Erzsébet tér (post-lunch)</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>13:55 (est.)</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>20 min</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>Walk Chain Bridge (~10 min, iconic Danube crossing) → Funicular up to Castle Hill (€6 one-way, ~5 min; or walk up ~15 min) | https://www.google.com/maps/dir/?api=1&amp;origin=V%C3%B6r%C3%B6smarty%20t%C3%A9r%2C%20Budapest&amp;destination=Buda%20Castle%2C%20Szent%20Gy%C3%B6rgy%20t%C3%A9r%202%2C%201014%20Budapest&amp;travelmode=walking</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Budapest</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Fisherman's Bastion + Matthias Church — Szentháromság tér, 1014 Budapest (the iconic skyline shot of Pest)</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>From: Buda Castle / Royal Palace courtyards</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>14:35 (est.)</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>Short walk; ~45-min visit. After: Tram 19 or 41 from Clark Ádám tér south to Déli (~10 min); ~1.5h buffer at Déli before 17:45 RJ 1068 to Vienna | https://www.google.com/maps/dir/?api=1&amp;origin=Buda%20Castle%2C%20Budapest&amp;destination=Fisherman%27s%20Bastion%2C%20Szenth%C3%A1roms%C3%A1g%20t%C3%A9r%2C%201014%20Budapest&amp;travelmode=walking</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>17:45</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>Budapest → Vienna</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
         <is>
           <t>Train</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F19" s="7" t="inlineStr">
         <is>
           <t>RegioJet RJ 1068 (same-day return)</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="G19" s="7" t="inlineStr">
         <is>
           <t>Budapest Déli — 17:45</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="H19" s="7" t="inlineStr">
         <is>
           <t>Vienna Central Train Station — 20:27</t>
         </is>
       </c>
-      <c r="I8" s="6" t="inlineStr">
+      <c r="I19" s="7" t="inlineStr">
         <is>
           <t>2h 42m</t>
         </is>
       </c>
-      <c r="J8" s="6" t="inlineStr">
+      <c r="J19" s="7" t="inlineStr">
         <is>
           <t>Trainline: https://app.trainline.com/MeSYEbQb12b</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Vienna (Option 1/4)</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Schönbrunn Palace &amp; Gardens — Schönbrunner Schloßstraße 47, 1130 Wien (UNESCO Habsburg residence; Gloriette views)</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>From: Margaretengürtel 6, 1050 Wien (Airbnb)</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>09:45 (est.)</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>15 min</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>U-Bahn U4 from Margaretengürtel → Schönbrunn (3 stops) | https://www.google.com/maps/dir/?api=1&amp;origin=Margareteng%C3%BCrtel%206%2C%201050%20Wien&amp;destination=Sch%C3%B6nbrunn%20Palace%2C%20Vienna&amp;travelmode=transit</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Vienna (Option 2/4)</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Hofburg complex + Albertina Museum — Heldenplatz/Albertinaplatz 1, 1010 Wien (Imperial Apartments interior, Sisi Museum, Treasury; Albertina art museum 2 min walk). Distinct from May 19 walking-tour exterior pass.</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>From: Margaretengürtel 6, 1050 Wien (Airbnb)</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>10:20 (est.)</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>20 min</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>U-Bahn U4 to Karlsplatz → walk 8 min | https://www.google.com/maps/dir/?api=1&amp;origin=Margareteng%C3%BCrtel%206%2C%201050%20Wien&amp;destination=Hofburg%2C%20Vienna&amp;travelmode=transit</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Vienna → Bratislava (Option 3/4)</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Day-trip to Bratislava, Slovakia — walkable Old Town + Bratislava Castle (~1h train each way; full day)</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>From: Margaretengürtel 6, 1050 Wien (Airbnb)</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>09:45 (est.)</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>1h 15m</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>Transit to Wien Hauptbahnhof → REX 1 train to Bratislava hl. st. (~1h) | https://www.google.com/maps/dir/?api=1&amp;origin=Margareteng%C3%BCrtel%206%2C%201050%20Wien&amp;destination=Bratislava%20hl.%20st.%2C%20Slovakia&amp;travelmode=transit</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Vienna → Melk (Option 4/4)</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Day-trip to Wachau Valley &amp; Melk Abbey — Stift Melk, 3390 Melk (Danube wine region; Baroque abbey; ~1h train + optional Danube boat)</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>From: Margaretengürtel 6, 1050 Wien (Airbnb)</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>09:15 (est.)</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>1h 15m</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>Transit to Wien Hauptbahnhof → ICE/RJ to Melk Bahnhof (~1h) | https://www.google.com/maps/dir/?api=1&amp;origin=Margareteng%C3%BCrtel%206%2C%201050%20Wien&amp;destination=Stift%20Melk%2C%20Melk&amp;travelmode=transit</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t>2026-05-22</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>06:39</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D24" s="7" t="inlineStr">
         <is>
           <t>Vienna → Prague</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E24" s="7" t="inlineStr">
         <is>
           <t>Train</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F24" s="7" t="inlineStr">
         <is>
           <t>RegioJet RJ 1030</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="G24" s="7" t="inlineStr">
         <is>
           <t>Vienna Central Train Station — 06:39</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="H24" s="7" t="inlineStr">
         <is>
           <t>Praha hl.n. — 10:56</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr">
+      <c r="I24" s="7" t="inlineStr">
         <is>
           <t>4h 17m</t>
         </is>
       </c>
-      <c r="J9" s="6" t="inlineStr">
+      <c r="J24" s="7" t="inlineStr">
         <is>
           <t>Trainline: https://app.trainline.com/K0MINBRb12b</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>2026-05-22</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr"/>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr"/>
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>Prague</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Tips</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>DPP 72-hour pass (250 CZK / ~€10) — metro + tram + bus; tap-and-pay also accepted on trams</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr"/>
+      <c r="H25" s="4" t="inlineStr"/>
+      <c r="I25" s="4" t="inlineStr"/>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>Attractions: Prague Visitor Pass (or CoolPass) bundles Castle + Jewish Museum + tower climbs; Prague Castle basic-loop ticket (~CZK 250); book Old-New Synagogue + Klementinum tour online | Explore: trdelník (touristy but iconic), goulash + knedlíky at U Medvídků, Pilsner Urquell beer, Charles Bridge at dawn (avoid crowds), Vinohrady neighbourhood cafés near Airbnb</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr"/>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>Prague</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
         <is>
           <t>Lodging (Airbnb)</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F26" s="6" t="inlineStr">
         <is>
           <t>Španělská 759/4, 120 00 Vinohrady, Czechia</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="G26" s="6" t="inlineStr">
         <is>
           <t>Check-in: 2026-05-22</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="H26" s="6" t="inlineStr">
         <is>
           <t>Check-out: 2026-05-26</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="I26" s="6" t="inlineStr">
         <is>
           <t>4 nights</t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="J26" s="6" t="inlineStr">
         <is>
           <t>Google Maps: https://maps.app.goo.gl/UcKWdy4NRJWvL3eZA</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>2026-05-23</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>08:31</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t>Prague → Dresden</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E27" s="7" t="inlineStr">
         <is>
           <t>Train</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F27" s="7" t="inlineStr">
         <is>
           <t>Deutsche Bahn 178 (day-trip outbound)</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="G27" s="7" t="inlineStr">
         <is>
           <t>Praha hl.n. — 08:31</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="H27" s="7" t="inlineStr">
         <is>
           <t>Dresden Hbf — 10:50</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr">
+      <c r="I27" s="7" t="inlineStr">
         <is>
           <t>2h 19m</t>
         </is>
       </c>
-      <c r="J11" s="6" t="inlineStr">
+      <c r="J27" s="7" t="inlineStr">
         <is>
           <t>Trainline: https://app.trainline.com/KXTU6ZSb12b</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>2026-05-23</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr"/>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Dresden</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>Tips</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>DVB 1-day ticket (~€8.20) for trams + buses; Old Town (Altstadt) is compact and walkable from Hbf via tram 8/9</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr"/>
+      <c r="H28" s="4" t="inlineStr"/>
+      <c r="I28" s="4" t="inlineStr"/>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>Attractions: Dresden Museums Day Card (€25) covers Zwinger + Albertinum + Royal Palace; Frauenkirche entry free (donation); pre-book Historic Green Vault timed-entry online (sells out) | Explore: Eierschecke cake, Saxon white wine, Zwinger Old Masters Picture Gallery (Raphael's Sistine Madonna), Brühl's Terrace ('Balcony of Europe') for Elbe views</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
         <is>
           <t>19:10</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D29" s="7" t="inlineStr">
         <is>
           <t>Dresden → Prague</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E29" s="7" t="inlineStr">
         <is>
           <t>Train</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="F29" s="7" t="inlineStr">
         <is>
           <t>Deutsche Bahn 385 (day-trip return)</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="G29" s="7" t="inlineStr">
         <is>
           <t>Dresden Hbf — 19:10</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="H29" s="7" t="inlineStr">
         <is>
           <t>Praha hl.n. — 21:25</t>
         </is>
       </c>
-      <c r="I12" s="6" t="inlineStr">
+      <c r="I29" s="7" t="inlineStr">
         <is>
           <t>2h 15m</t>
         </is>
       </c>
-      <c r="J12" s="6" t="inlineStr">
+      <c r="J29" s="7" t="inlineStr">
         <is>
           <t>Trainline: https://app.trainline.com/Uo4dOhUb12b</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>2026-05-26</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>Tue</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>Prague → Stockholm</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>Flight</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Norwegian D82621 (Norwegian Air Sweden AOC AB); Ticket type: LOWFARE+; Seat 12C; Baggage: 1 checked + 1 underseat + 1 overhead</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>Prague Václav Havel (PRG), Terminal 2 — 12:10</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>Stockholm Arlanda (ARN), Terminal 5 — 14:05</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="I30" s="2" t="inlineStr">
         <is>
           <t>1h 55m</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J30" s="2" t="inlineStr">
         <is>
           <t>Booking ref: Y9GHBZ; Ticket: 328 2404310661 (Norwegian Air Manolet.pdf)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>2026-05-26</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>Tue</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr"/>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr"/>
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>Stockholm</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>Tips</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>SL Access 72-hour pass (~SEK 295 / €26) — metro + tram + bus + commuter ferry; airport: Arlanda Express train (~SEK 320 / €28, 18 min) or SL commuter rail (cheaper, ~40 min)</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr"/>
+      <c r="H31" s="4" t="inlineStr"/>
+      <c r="I31" s="4" t="inlineStr"/>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>Attractions: Vasa Museum (~SEK 220) is the single best stop; Skansen open-air museum + Royal Palace; Go City Stockholm Pass for heavy sightseeing | Explore: fika culture (coffee + kanelbulle cinnamon bun), Swedish meatballs at Pelikan or Tradition, Gamla Stan cobbled Old Town, Södermalm hipster cafés near hotel, archipelago boat from Strömkajen</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr"/>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>Stockholm</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
         <is>
           <t>Lodging (Hotel)</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F32" s="6" t="inlineStr">
         <is>
           <t>Bob W Stockholm Södermalm</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G32" s="6" t="inlineStr">
         <is>
           <t>Check-in: 2026-05-26</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H32" s="6" t="inlineStr">
         <is>
           <t>Check-out: 2026-05-30</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="I32" s="6" t="inlineStr">
         <is>
           <t>4 nights</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="J32" s="6" t="inlineStr">
         <is>
           <t>Google Maps: https://maps.app.goo.gl/QzqTafk4EjpTVc577</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>2026-05-30</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr"/>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr"/>
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>Stockholm → Istanbul</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>Flight</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>Flight J1796</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>Stockholm Arlanda Airport</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>Istanbul</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr"/>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="I33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr">
         <is>
           <t>Transfer to Stockholm Arlanda; departure from Schengen area; in-flight overnight</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>2026-05-31</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>Istanbul → Manila</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>Flight</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Flight J0084</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>Istanbul</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>Manila</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr"/>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="I34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr">
         <is>
           <t>Return flight to Manila</t>
         </is>

</xml_diff>